<commit_message>
R4.5 rev. ANL: sin nodos sueltos, espectro recalibrado, 100 modos
- Se quitan los nodos 225-232 sin miembros (origen de los ~460 warnings
  de rigidez cero en el .ANL)
- Factores de SPECTRUM con el .ANL R4.5: X 1.1599 (antes 1.5377),
  Z 2.0938 (antes 2.7081); CUT OFF MODE SHAPE 100 porque Z quedo en
  89.745% con 50 modos
- EspectrosSismo y AreasTributarias con T, W dinamico y V SRSS del .ANL;
  V minimo como formula
- Peso y desglose con la participacion y factores nuevos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DbpSpoM7qi5cJ9LMKpwgVv
</commit_message>
<xml_diff>
--- a/R4.5/AreasTributarias_NOSE_DOCK_H5_H6_R4.5.xlsx
+++ b/R4.5/AreasTributarias_NOSE_DOCK_H5_H6_R4.5.xlsx
@@ -2182,10 +2182,10 @@
     <t xml:space="preserve">W dinámico de STAAD — dirección X</t>
   </si>
   <si>
-    <t xml:space="preserve">DYNAMIC WEIGHT del análisis modal (R4.4). Correr R4.5 y capturar aquí el nuevo valor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.ANL R4.4 — PENDIENTE .ANL R4.5</t>
+    <t xml:space="preserve">DYNAMIC WEIGHT del análisis modal R4.5 (igual en X y Z).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.ANL R4.5</t>
   </si>
   <si>
     <t xml:space="preserve">5. CORTANTE MÍNIMO NTDS §5.4.1(3) → FACTOR DEL SPECTRUM EN STAAD</t>
@@ -2245,13 +2245,13 @@
     <t xml:space="preserve">T_B en X (modo con más masa en X)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 3: mayor participación en X.</t>
+    <t xml:space="preserve">Modo 1: mayor participación en X.</t>
   </si>
   <si>
     <t xml:space="preserve">T_B en Z (modo con más masa en Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">Modo 30: mayor participación en Z.</t>
+    <t xml:space="preserve">Modo 14: mayor participación en Z.</t>
   </si>
   <si>
     <t xml:space="preserve">V_est en X = máx(Cs(T_B), 0.8·Cs(T_A))·W</t>
@@ -2312,6 +2312,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2517,136 +2518,140 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="12" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -10241,48 +10246,48 @@
       <c r="S93" s="10" t="s">
         <v>456</v>
       </c>
-      <c r="T93" s="0"/>
-      <c r="U93" s="0"/>
-      <c r="V93" s="0"/>
-      <c r="W93" s="0"/>
-      <c r="X93" s="0"/>
-      <c r="Y93" s="0"/>
-      <c r="Z93" s="0"/>
-      <c r="AA93" s="0"/>
-      <c r="AB93" s="0"/>
-      <c r="AC93" s="0"/>
-      <c r="AD93" s="0"/>
-      <c r="AE93" s="0"/>
-      <c r="AF93" s="0"/>
-      <c r="AG93" s="0"/>
-      <c r="AH93" s="0"/>
-      <c r="AI93" s="0"/>
-      <c r="AJ93" s="0"/>
-      <c r="AK93" s="0"/>
-      <c r="AL93" s="0"/>
-      <c r="AM93" s="0"/>
-      <c r="AN93" s="0"/>
-      <c r="AO93" s="0"/>
-      <c r="AP93" s="0"/>
-      <c r="AQ93" s="0"/>
-      <c r="AR93" s="0"/>
-      <c r="AS93" s="0"/>
-      <c r="AT93" s="0"/>
-      <c r="AU93" s="0"/>
-      <c r="AV93" s="0"/>
-      <c r="AW93" s="0"/>
-      <c r="AX93" s="0"/>
-      <c r="AY93" s="0"/>
-      <c r="AZ93" s="0"/>
-      <c r="BA93" s="0"/>
-      <c r="BB93" s="0"/>
-      <c r="BC93" s="0"/>
-      <c r="BD93" s="0"/>
-      <c r="BE93" s="0"/>
-      <c r="BF93" s="0"/>
-      <c r="BG93" s="0"/>
-      <c r="BH93" s="0"/>
-      <c r="BI93" s="0"/>
+      <c r="T93" s="29"/>
+      <c r="U93" s="29"/>
+      <c r="V93" s="29"/>
+      <c r="W93" s="29"/>
+      <c r="X93" s="29"/>
+      <c r="Y93" s="29"/>
+      <c r="Z93" s="29"/>
+      <c r="AA93" s="29"/>
+      <c r="AB93" s="29"/>
+      <c r="AC93" s="29"/>
+      <c r="AD93" s="29"/>
+      <c r="AE93" s="29"/>
+      <c r="AF93" s="29"/>
+      <c r="AG93" s="29"/>
+      <c r="AH93" s="29"/>
+      <c r="AI93" s="29"/>
+      <c r="AJ93" s="29"/>
+      <c r="AK93" s="29"/>
+      <c r="AL93" s="29"/>
+      <c r="AM93" s="29"/>
+      <c r="AN93" s="29"/>
+      <c r="AO93" s="29"/>
+      <c r="AP93" s="29"/>
+      <c r="AQ93" s="29"/>
+      <c r="AR93" s="29"/>
+      <c r="AS93" s="29"/>
+      <c r="AT93" s="29"/>
+      <c r="AU93" s="29"/>
+      <c r="AV93" s="29"/>
+      <c r="AW93" s="29"/>
+      <c r="AX93" s="29"/>
+      <c r="AY93" s="29"/>
+      <c r="AZ93" s="29"/>
+      <c r="BA93" s="29"/>
+      <c r="BB93" s="29"/>
+      <c r="BC93" s="29"/>
+      <c r="BD93" s="29"/>
+      <c r="BE93" s="29"/>
+      <c r="BF93" s="29"/>
+      <c r="BG93" s="29"/>
+      <c r="BH93" s="29"/>
+      <c r="BI93" s="29"/>
     </row>
     <row r="94" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="21" t="s">
@@ -14136,11 +14141,11 @@
       <c r="F95" s="21"/>
     </row>
     <row r="97" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B97" s="29"/>
-      <c r="C97" s="29"/>
-      <c r="D97" s="29"/>
-      <c r="E97" s="29"/>
-      <c r="F97" s="29"/>
+      <c r="B97" s="30"/>
+      <c r="C97" s="30"/>
+      <c r="D97" s="30"/>
+      <c r="E97" s="30"/>
+      <c r="F97" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -14430,12 +14435,12 @@
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="31" t="s">
         <v>669</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="32" t="s">
         <v>670</v>
       </c>
     </row>
@@ -14463,7 +14468,7 @@
       <c r="C23" s="7" t="n">
         <v>40.06</v>
       </c>
-      <c r="D23" s="32" t="n">
+      <c r="D23" s="33" t="n">
         <v>34.6451</v>
       </c>
       <c r="E23" s="19" t="n">
@@ -14480,7 +14485,7 @@
       <c r="C24" s="7" t="n">
         <v>19.8225</v>
       </c>
-      <c r="D24" s="32" t="n">
+      <c r="D24" s="33" t="n">
         <v>57.8063</v>
       </c>
       <c r="E24" s="19" t="n">
@@ -14497,7 +14502,7 @@
       <c r="C25" s="7" t="n">
         <v>30.24</v>
       </c>
-      <c r="D25" s="32" t="n">
+      <c r="D25" s="33" t="n">
         <v>16.5577</v>
       </c>
       <c r="E25" s="19" t="n">
@@ -14514,7 +14519,7 @@
       <c r="C26" s="7" t="n">
         <v>32.043</v>
       </c>
-      <c r="D26" s="32" t="n">
+      <c r="D26" s="33" t="n">
         <v>25.81</v>
       </c>
       <c r="E26" s="19" t="n">
@@ -14531,7 +14536,7 @@
       <c r="C27" s="7" t="n">
         <v>42.08</v>
       </c>
-      <c r="D27" s="32" t="n">
+      <c r="D27" s="33" t="n">
         <v>18.4851</v>
       </c>
       <c r="E27" s="19" t="n">
@@ -14548,7 +14553,7 @@
       <c r="C28" s="7" t="n">
         <v>140</v>
       </c>
-      <c r="D28" s="32" t="n">
+      <c r="D28" s="33" t="n">
         <v>12.905</v>
       </c>
       <c r="E28" s="19" t="n">
@@ -14565,7 +14570,7 @@
       <c r="C29" s="7" t="n">
         <v>110.88</v>
       </c>
-      <c r="D29" s="32" t="n">
+      <c r="D29" s="33" t="n">
         <v>9.2425</v>
       </c>
       <c r="E29" s="19" t="n">
@@ -14582,7 +14587,7 @@
       <c r="C30" s="7" t="n">
         <v>84</v>
       </c>
-      <c r="D30" s="32" t="n">
+      <c r="D30" s="33" t="n">
         <v>6.3515</v>
       </c>
       <c r="E30" s="19" t="n">
@@ -14599,7 +14604,7 @@
       <c r="C31" s="7" t="n">
         <v>23.68</v>
       </c>
-      <c r="D31" s="32" t="n">
+      <c r="D31" s="33" t="n">
         <v>3.9423</v>
       </c>
       <c r="E31" s="19" t="n">
@@ -14616,7 +14621,7 @@
       <c r="C32" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D32" s="32" t="n">
+      <c r="D32" s="33" t="n">
         <v>8.3872</v>
       </c>
       <c r="E32" s="19" t="n">
@@ -14633,7 +14638,7 @@
       <c r="C33" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="D33" s="32" t="n">
+      <c r="D33" s="33" t="n">
         <v>17.4193</v>
       </c>
       <c r="E33" s="19" t="n">
@@ -14650,7 +14655,7 @@
       <c r="C34" s="7" t="n">
         <v>64.0861</v>
       </c>
-      <c r="D34" s="32" t="n">
+      <c r="D34" s="33" t="n">
         <v>2.0129</v>
       </c>
       <c r="E34" s="19" t="n">
@@ -14667,7 +14672,7 @@
       <c r="C35" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="D35" s="32" t="n">
+      <c r="D35" s="33" t="n">
         <v>1.5097</v>
       </c>
       <c r="E35" s="19" t="n">
@@ -14684,7 +14689,7 @@
       <c r="C36" s="7" t="n">
         <v>173.5764</v>
       </c>
-      <c r="D36" s="32" t="n">
+      <c r="D36" s="33" t="n">
         <v>5.0671</v>
       </c>
       <c r="E36" s="19" t="n">
@@ -14717,7 +14722,7 @@
       <c r="F38" s="10"/>
     </row>
     <row r="39" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="30" t="s">
+      <c r="B39" s="31" t="s">
         <v>701</v>
       </c>
     </row>
@@ -14850,7 +14855,7 @@
         <v>717</v>
       </c>
       <c r="C47" s="11" t="n">
-        <v>13.15704</v>
+        <v>13.10796</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>703</v>
@@ -14870,7 +14875,7 @@
       <c r="F48" s="10"/>
     </row>
     <row r="49" s="1" customFormat="true" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="30" t="s">
+      <c r="B49" s="31" t="s">
         <v>720</v>
       </c>
     </row>
@@ -15052,7 +15057,7 @@
         <v>738</v>
       </c>
       <c r="C60" s="11" t="n">
-        <v>0.36976</v>
+        <v>0.78665</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>727</v>
@@ -15069,7 +15074,7 @@
         <v>740</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>0.12899</v>
+        <v>0.1782</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>727</v>
@@ -15086,7 +15091,8 @@
         <v>742</v>
       </c>
       <c r="C62" s="11" t="n">
-        <v>2255.49257142857</v>
+        <f aca="false">MAX(C51*C52*C53/C55*(C54/MAX(C60,C54))^(2/3),0.8*C59)*C47*1000</f>
+        <v>1875.85003499262</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>58</v>
@@ -15103,7 +15109,8 @@
         <v>744</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>2254.57542857143</v>
+        <f aca="false">MAX(C51*C52*C53/C55*(C54/MAX(C61,C54))^(2/3),0.8*C59)*C47*1000</f>
+        <v>2247.07885714286</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>58</v>
@@ -15120,7 +15127,8 @@
         <v>745</v>
       </c>
       <c r="C64" s="11" t="n">
-        <v>2029.94331428571</v>
+        <f aca="false">MAX(0.9*C62,0.8*C59*C47*1000)</f>
+        <v>1797.66308571429</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>58</v>
@@ -15137,7 +15145,8 @@
         <v>747</v>
       </c>
       <c r="C65" s="11" t="n">
-        <v>2029.11788571429</v>
+        <f aca="false">MAX(0.9*C63,0.8*C59*C47*1000)</f>
+        <v>2022.37097142857</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>58</v>
@@ -15154,7 +15163,7 @@
         <v>748</v>
       </c>
       <c r="C66" s="11" t="n">
-        <v>1320.0862927315</v>
+        <v>1549.83416791312</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>58</v>
@@ -15171,7 +15180,7 @@
         <v>750</v>
       </c>
       <c r="C67" s="11" t="n">
-        <v>749.264900662252</v>
+        <v>965.872752114028</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>58</v>
@@ -15189,7 +15198,7 @@
       </c>
       <c r="C68" s="11" t="n">
         <f aca="false">MAX(1,C64/C66)</f>
-        <v>1.53773531735217</v>
+        <v>1.15990673256022</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>41</v>
@@ -15207,7 +15216,7 @@
       </c>
       <c r="C69" s="11" t="n">
         <f aca="false">MAX(1,C65/C67)</f>
-        <v>2.70814485493824</v>
+        <v>2.09382754301968</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>41</v>

</xml_diff>